<commit_message>
fix: corrigir coordenadas da UBS Faveira em Passagem Franca
Atualiza lat/lng para -6.188648, -43.780340 na planilha modelo.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/templates/banco_localizacoes_ubs.xlsx
+++ b/docs/templates/banco_localizacoes_ubs.xlsx
@@ -550,13 +550,13 @@
         <v>Urbana</v>
       </c>
       <c r="C9">
-        <v>-3.531601</v>
+        <v>-6.188648</v>
       </c>
       <c r="D9">
-        <v>-41.63003</v>
+        <v>-43.78034</v>
       </c>
       <c r="E9" t="str">
-        <v>-3.531601, -41.63003</v>
+        <v>-6.188648, -43.78034</v>
       </c>
     </row>
     <row r="10">

</xml_diff>